<commit_message>
090225 - updated format/font size in week 16 skins - get all data on single page
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 16 Skins.xlsx
+++ b/public/results/2025/Week 16 Skins.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B45FE0E-8E6F-1747-99E0-4FE6244FB248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{2B45FE0E-8E6F-1747-99E0-4FE6244FB248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{172882C6-DD7E-42F9-9429-71C145409A3C}"/>
   <bookViews>
-    <workbookView xWindow="6860" yWindow="700" windowWidth="31360" windowHeight="17120" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
+    <workbookView xWindow="4515" yWindow="1545" windowWidth="30765" windowHeight="17115" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 16 Skins" sheetId="1" r:id="rId1"/>
@@ -126,7 +126,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,29 +172,23 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="22"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="22"/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -585,7 +579,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -704,20 +698,26 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
@@ -728,26 +728,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1085,32 +1073,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F8EC831-685C-42E6-9510-7BA05FCAF636}">
   <dimension ref="A1:O36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="6.5" style="4" customWidth="1"/>
-    <col min="3" max="11" width="8.6640625" style="4" customWidth="1"/>
-    <col min="12" max="12" width="3.1640625" style="4" customWidth="1"/>
-    <col min="13" max="13" width="5.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.33203125" style="4" customWidth="1"/>
-    <col min="15" max="15" width="6.83203125" style="4" customWidth="1"/>
-    <col min="16" max="16384" width="9.1640625" style="4"/>
+    <col min="1" max="1" width="8.140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" style="4" customWidth="1"/>
+    <col min="3" max="11" width="8.7109375" style="4" customWidth="1"/>
+    <col min="12" max="12" width="3.140625" style="4" customWidth="1"/>
+    <col min="13" max="13" width="5.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.28515625" style="4" customWidth="1"/>
+    <col min="15" max="15" width="6.85546875" style="4" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="43" t="s">
+    <row r="1" spans="1:15" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
       <c r="L1" s="20"/>
       <c r="M1" s="21" t="s">
         <v>0</v>
@@ -1120,7 +1108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
         <v>2</v>
       </c>
@@ -1154,14 +1142,14 @@
       <c r="K2" s="25">
         <v>9</v>
       </c>
-      <c r="L2" s="45" t="s">
+      <c r="L2" s="47" t="s">
         <v>5</v>
       </c>
       <c r="M2" s="6"/>
       <c r="N2" s="7"/>
       <c r="O2" s="8"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="26"/>
       <c r="B3" s="27" t="s">
         <v>4</v>
@@ -1193,12 +1181,12 @@
       <c r="K3" s="28">
         <v>5</v>
       </c>
-      <c r="L3" s="46"/>
+      <c r="L3" s="48"/>
       <c r="M3" s="9"/>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
     </row>
-    <row r="4" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="29"/>
       <c r="B4" s="30" t="s">
         <v>5</v>
@@ -1230,43 +1218,43 @@
       <c r="K4" s="31">
         <v>2</v>
       </c>
-      <c r="L4" s="47"/>
+      <c r="L4" s="49"/>
       <c r="M4" s="15"/>
       <c r="N4" s="16"/>
       <c r="O4" s="16"/>
     </row>
-    <row r="5" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="40">
-        <v>6</v>
-      </c>
-      <c r="D5" s="40">
+      <c r="C5" s="1">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1">
         <v>8</v>
       </c>
-      <c r="E5" s="40">
-        <v>6</v>
-      </c>
-      <c r="F5" s="40">
-        <v>4</v>
-      </c>
-      <c r="G5" s="40">
-        <v>5</v>
-      </c>
-      <c r="H5" s="40">
-        <v>5</v>
-      </c>
-      <c r="I5" s="40">
-        <v>6</v>
-      </c>
-      <c r="J5" s="40">
+      <c r="E5" s="1">
+        <v>6</v>
+      </c>
+      <c r="F5" s="1">
+        <v>4</v>
+      </c>
+      <c r="G5" s="1">
+        <v>5</v>
+      </c>
+      <c r="H5" s="1">
+        <v>5</v>
+      </c>
+      <c r="I5" s="1">
+        <v>6</v>
+      </c>
+      <c r="J5" s="1">
         <v>7</v>
       </c>
-      <c r="K5" s="40">
+      <c r="K5" s="1">
         <v>8</v>
       </c>
       <c r="L5" s="33"/>
@@ -1274,36 +1262,36 @@
       <c r="N5" s="18"/>
       <c r="O5" s="7"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="34"/>
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="48">
-        <v>3</v>
-      </c>
-      <c r="D6" s="48">
-        <v>3</v>
-      </c>
-      <c r="E6" s="48">
-        <v>3</v>
-      </c>
-      <c r="F6" s="48">
-        <v>2</v>
-      </c>
-      <c r="G6" s="48">
-        <v>3</v>
-      </c>
-      <c r="H6" s="48">
-        <v>2</v>
-      </c>
-      <c r="I6" s="48">
-        <v>2</v>
-      </c>
-      <c r="J6" s="48">
-        <v>2</v>
-      </c>
-      <c r="K6" s="49">
+      <c r="C6" s="41">
+        <v>3</v>
+      </c>
+      <c r="D6" s="41">
+        <v>3</v>
+      </c>
+      <c r="E6" s="41">
+        <v>3</v>
+      </c>
+      <c r="F6" s="41">
+        <v>2</v>
+      </c>
+      <c r="G6" s="41">
+        <v>3</v>
+      </c>
+      <c r="H6" s="41">
+        <v>2</v>
+      </c>
+      <c r="I6" s="41">
+        <v>2</v>
+      </c>
+      <c r="J6" s="41">
+        <v>2</v>
+      </c>
+      <c r="K6" s="42">
         <v>3</v>
       </c>
       <c r="L6" s="35">
@@ -1314,7 +1302,7 @@
       <c r="N6" s="12"/>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="36"/>
       <c r="B7" s="3" t="s">
         <v>8</v>
@@ -1323,7 +1311,7 @@
         <f>C5-C6</f>
         <v>3</v>
       </c>
-      <c r="D7" s="50">
+      <c r="D7" s="43">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
         <v>5</v>
       </c>
@@ -1343,15 +1331,15 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="I7" s="50">
+      <c r="I7" s="43">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="J7" s="50">
+      <c r="J7" s="43">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K7" s="51">
+      <c r="K7" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1366,38 +1354,38 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="32" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="40">
-        <v>5</v>
-      </c>
-      <c r="D8" s="40">
+      <c r="C8" s="1">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1">
         <v>7</v>
       </c>
-      <c r="E8" s="40">
-        <v>5</v>
-      </c>
-      <c r="F8" s="40">
-        <v>6</v>
-      </c>
-      <c r="G8" s="40">
-        <v>5</v>
-      </c>
-      <c r="H8" s="40">
+      <c r="E8" s="1">
+        <v>5</v>
+      </c>
+      <c r="F8" s="1">
+        <v>6</v>
+      </c>
+      <c r="G8" s="1">
+        <v>5</v>
+      </c>
+      <c r="H8" s="1">
         <v>7</v>
       </c>
-      <c r="I8" s="40">
-        <v>4</v>
-      </c>
-      <c r="J8" s="40">
-        <v>4</v>
-      </c>
-      <c r="K8" s="40">
+      <c r="I8" s="1">
+        <v>4</v>
+      </c>
+      <c r="J8" s="1">
+        <v>4</v>
+      </c>
+      <c r="K8" s="1">
         <v>5</v>
       </c>
       <c r="L8" s="33"/>
@@ -1405,36 +1393,36 @@
       <c r="N8" s="18"/>
       <c r="O8" s="7"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="34"/>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="48">
-        <v>2</v>
-      </c>
-      <c r="D9" s="48">
-        <v>2</v>
-      </c>
-      <c r="E9" s="48">
-        <v>2</v>
-      </c>
-      <c r="F9" s="48">
-        <v>1</v>
-      </c>
-      <c r="G9" s="48">
-        <v>1</v>
-      </c>
-      <c r="H9" s="48">
-        <v>1</v>
-      </c>
-      <c r="I9" s="48">
-        <v>1</v>
-      </c>
-      <c r="J9" s="48">
-        <v>1</v>
-      </c>
-      <c r="K9" s="49">
+      <c r="C9" s="41">
+        <v>2</v>
+      </c>
+      <c r="D9" s="41">
+        <v>2</v>
+      </c>
+      <c r="E9" s="41">
+        <v>2</v>
+      </c>
+      <c r="F9" s="41">
+        <v>1</v>
+      </c>
+      <c r="G9" s="41">
+        <v>1</v>
+      </c>
+      <c r="H9" s="41">
+        <v>1</v>
+      </c>
+      <c r="I9" s="41">
+        <v>1</v>
+      </c>
+      <c r="J9" s="41">
+        <v>1</v>
+      </c>
+      <c r="K9" s="42">
         <v>2</v>
       </c>
       <c r="L9" s="35">
@@ -1445,7 +1433,7 @@
       <c r="N9" s="12"/>
       <c r="O9" s="10"/>
     </row>
-    <row r="10" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="36"/>
       <c r="B10" s="3" t="s">
         <v>8</v>
@@ -1454,7 +1442,7 @@
         <f>C8-C9</f>
         <v>3</v>
       </c>
-      <c r="D10" s="50">
+      <c r="D10" s="43">
         <f t="shared" ref="D10:K10" si="1">D8-D9</f>
         <v>5</v>
       </c>
@@ -1462,19 +1450,19 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="F10" s="50">
+      <c r="F10" s="43">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="G10" s="50">
+      <c r="G10" s="43">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="H10" s="50">
+      <c r="H10" s="43">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="I10" s="50">
+      <c r="I10" s="43">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -1482,7 +1470,7 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="K10" s="53">
+      <c r="K10" s="45">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -1491,38 +1479,38 @@
       <c r="N10" s="19"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="32" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="40">
-        <v>6</v>
-      </c>
-      <c r="D11" s="40">
-        <v>6</v>
-      </c>
-      <c r="E11" s="40">
+      <c r="C11" s="1">
+        <v>6</v>
+      </c>
+      <c r="D11" s="1">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1">
         <v>7</v>
       </c>
-      <c r="F11" s="40">
-        <v>4</v>
-      </c>
-      <c r="G11" s="40">
-        <v>4</v>
-      </c>
-      <c r="H11" s="40">
+      <c r="F11" s="1">
+        <v>4</v>
+      </c>
+      <c r="G11" s="1">
+        <v>4</v>
+      </c>
+      <c r="H11" s="1">
         <v>7</v>
       </c>
-      <c r="I11" s="40">
-        <v>4</v>
-      </c>
-      <c r="J11" s="40">
+      <c r="I11" s="1">
+        <v>4</v>
+      </c>
+      <c r="J11" s="1">
         <v>7</v>
       </c>
-      <c r="K11" s="40">
+      <c r="K11" s="1">
         <v>6</v>
       </c>
       <c r="L11" s="35"/>
@@ -1530,36 +1518,36 @@
       <c r="N11" s="18"/>
       <c r="O11" s="7"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="34"/>
       <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="48">
-        <v>1</v>
-      </c>
-      <c r="D12" s="48">
-        <v>2</v>
-      </c>
-      <c r="E12" s="48">
-        <v>2</v>
-      </c>
-      <c r="F12" s="48">
-        <v>1</v>
-      </c>
-      <c r="G12" s="48">
-        <v>1</v>
-      </c>
-      <c r="H12" s="48">
-        <v>1</v>
-      </c>
-      <c r="I12" s="48">
-        <v>1</v>
-      </c>
-      <c r="J12" s="48">
-        <v>1</v>
-      </c>
-      <c r="K12" s="49">
+      <c r="C12" s="41">
+        <v>1</v>
+      </c>
+      <c r="D12" s="41">
+        <v>2</v>
+      </c>
+      <c r="E12" s="41">
+        <v>2</v>
+      </c>
+      <c r="F12" s="41">
+        <v>1</v>
+      </c>
+      <c r="G12" s="41">
+        <v>1</v>
+      </c>
+      <c r="H12" s="41">
+        <v>1</v>
+      </c>
+      <c r="I12" s="41">
+        <v>1</v>
+      </c>
+      <c r="J12" s="41">
+        <v>1</v>
+      </c>
+      <c r="K12" s="42">
         <v>2</v>
       </c>
       <c r="L12" s="35">
@@ -1570,44 +1558,44 @@
       <c r="N12" s="12"/>
       <c r="O12" s="10"/>
     </row>
-    <row r="13" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="36"/>
       <c r="B13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="50">
+      <c r="C13" s="43">
         <f>C11-C12</f>
         <v>5</v>
       </c>
-      <c r="D13" s="50">
+      <c r="D13" s="43">
         <f t="shared" ref="D13:K13" si="2">D11-D12</f>
         <v>4</v>
       </c>
-      <c r="E13" s="50">
+      <c r="E13" s="43">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="F13" s="50">
+      <c r="F13" s="43">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="G13" s="50">
+      <c r="G13" s="43">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="H13" s="50">
+      <c r="H13" s="43">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="I13" s="50">
+      <c r="I13" s="43">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="J13" s="50">
+      <c r="J13" s="43">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="K13" s="50">
+      <c r="K13" s="43">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
@@ -1616,38 +1604,38 @@
       <c r="N13" s="19"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="32" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="40">
-        <v>6</v>
-      </c>
-      <c r="D14" s="40">
-        <v>5</v>
-      </c>
-      <c r="E14" s="40">
+      <c r="C14" s="1">
+        <v>6</v>
+      </c>
+      <c r="D14" s="1">
+        <v>5</v>
+      </c>
+      <c r="E14" s="1">
         <v>7</v>
       </c>
-      <c r="F14" s="40">
-        <v>5</v>
-      </c>
-      <c r="G14" s="40">
-        <v>5</v>
-      </c>
-      <c r="H14" s="40">
-        <v>6</v>
-      </c>
-      <c r="I14" s="40">
-        <v>4</v>
-      </c>
-      <c r="J14" s="40">
-        <v>6</v>
-      </c>
-      <c r="K14" s="40">
+      <c r="F14" s="1">
+        <v>5</v>
+      </c>
+      <c r="G14" s="1">
+        <v>5</v>
+      </c>
+      <c r="H14" s="1">
+        <v>6</v>
+      </c>
+      <c r="I14" s="1">
+        <v>4</v>
+      </c>
+      <c r="J14" s="1">
+        <v>6</v>
+      </c>
+      <c r="K14" s="1">
         <v>8</v>
       </c>
       <c r="L14" s="35"/>
@@ -1655,36 +1643,36 @@
       <c r="N14" s="18"/>
       <c r="O14" s="7"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="34"/>
       <c r="B15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="48">
-        <v>2</v>
-      </c>
-      <c r="D15" s="48">
-        <v>2</v>
-      </c>
-      <c r="E15" s="48">
-        <v>2</v>
-      </c>
-      <c r="F15" s="48">
-        <v>2</v>
-      </c>
-      <c r="G15" s="48">
-        <v>2</v>
-      </c>
-      <c r="H15" s="48">
-        <v>2</v>
-      </c>
-      <c r="I15" s="48">
-        <v>2</v>
-      </c>
-      <c r="J15" s="48">
-        <v>2</v>
-      </c>
-      <c r="K15" s="49">
+      <c r="C15" s="41">
+        <v>2</v>
+      </c>
+      <c r="D15" s="41">
+        <v>2</v>
+      </c>
+      <c r="E15" s="41">
+        <v>2</v>
+      </c>
+      <c r="F15" s="41">
+        <v>2</v>
+      </c>
+      <c r="G15" s="41">
+        <v>2</v>
+      </c>
+      <c r="H15" s="41">
+        <v>2</v>
+      </c>
+      <c r="I15" s="41">
+        <v>2</v>
+      </c>
+      <c r="J15" s="41">
+        <v>2</v>
+      </c>
+      <c r="K15" s="42">
         <v>2</v>
       </c>
       <c r="L15" s="35">
@@ -1695,12 +1683,12 @@
       <c r="N15" s="12"/>
       <c r="O15" s="10"/>
     </row>
-    <row r="16" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="36"/>
       <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="50">
+      <c r="C16" s="43">
         <f>C14-C15</f>
         <v>4</v>
       </c>
@@ -1708,31 +1696,31 @@
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
         <v>3</v>
       </c>
-      <c r="E16" s="50">
+      <c r="E16" s="43">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="F16" s="50">
+      <c r="F16" s="43">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="G16" s="50">
+      <c r="G16" s="43">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="H16" s="50">
+      <c r="H16" s="43">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="I16" s="50">
+      <c r="I16" s="43">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="J16" s="50">
+      <c r="J16" s="43">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="K16" s="50">
+      <c r="K16" s="43">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
@@ -1747,38 +1735,38 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="32" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="40">
-        <v>6</v>
-      </c>
-      <c r="D17" s="40">
-        <v>6</v>
-      </c>
-      <c r="E17" s="40">
-        <v>5</v>
-      </c>
-      <c r="F17" s="40">
-        <v>4</v>
-      </c>
-      <c r="G17" s="40">
+      <c r="C17" s="1">
+        <v>6</v>
+      </c>
+      <c r="D17" s="1">
+        <v>6</v>
+      </c>
+      <c r="E17" s="1">
+        <v>5</v>
+      </c>
+      <c r="F17" s="1">
+        <v>4</v>
+      </c>
+      <c r="G17" s="1">
         <v>7</v>
       </c>
-      <c r="H17" s="40">
-        <v>5</v>
-      </c>
-      <c r="I17" s="40">
-        <v>4</v>
-      </c>
-      <c r="J17" s="40">
-        <v>6</v>
-      </c>
-      <c r="K17" s="40">
+      <c r="H17" s="1">
+        <v>5</v>
+      </c>
+      <c r="I17" s="1">
+        <v>4</v>
+      </c>
+      <c r="J17" s="1">
+        <v>6</v>
+      </c>
+      <c r="K17" s="1">
         <v>5</v>
       </c>
       <c r="L17" s="35"/>
@@ -1786,36 +1774,36 @@
       <c r="N17" s="18"/>
       <c r="O17" s="7"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="34"/>
       <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="48">
-        <v>1</v>
-      </c>
-      <c r="D18" s="48">
-        <v>2</v>
-      </c>
-      <c r="E18" s="48">
-        <v>1</v>
-      </c>
-      <c r="F18" s="48">
-        <v>1</v>
-      </c>
-      <c r="G18" s="48">
-        <v>1</v>
-      </c>
-      <c r="H18" s="48">
-        <v>1</v>
-      </c>
-      <c r="I18" s="48">
-        <v>1</v>
-      </c>
-      <c r="J18" s="48">
-        <v>1</v>
-      </c>
-      <c r="K18" s="49">
+      <c r="C18" s="41">
+        <v>1</v>
+      </c>
+      <c r="D18" s="41">
+        <v>2</v>
+      </c>
+      <c r="E18" s="41">
+        <v>1</v>
+      </c>
+      <c r="F18" s="41">
+        <v>1</v>
+      </c>
+      <c r="G18" s="41">
+        <v>1</v>
+      </c>
+      <c r="H18" s="41">
+        <v>1</v>
+      </c>
+      <c r="I18" s="41">
+        <v>1</v>
+      </c>
+      <c r="J18" s="41">
+        <v>1</v>
+      </c>
+      <c r="K18" s="42">
         <v>2</v>
       </c>
       <c r="L18" s="35">
@@ -1826,40 +1814,40 @@
       <c r="N18" s="12"/>
       <c r="O18" s="10"/>
     </row>
-    <row r="19" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="36"/>
       <c r="B19" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="50">
+      <c r="C19" s="43">
         <f>C17-C18</f>
         <v>5</v>
       </c>
-      <c r="D19" s="50">
+      <c r="D19" s="43">
         <f t="shared" ref="D19:K19" si="4">D17-D18</f>
         <v>4</v>
       </c>
-      <c r="E19" s="50">
+      <c r="E19" s="43">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="F19" s="50">
+      <c r="F19" s="43">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="G19" s="50">
+      <c r="G19" s="43">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="H19" s="50">
+      <c r="H19" s="43">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="I19" s="50">
+      <c r="I19" s="43">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="J19" s="50">
+      <c r="J19" s="43">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
@@ -1872,38 +1860,38 @@
       <c r="N19" s="19"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="32" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="40">
-        <v>5</v>
-      </c>
-      <c r="D20" s="40">
+      <c r="C20" s="1">
+        <v>5</v>
+      </c>
+      <c r="D20" s="1">
         <v>7</v>
       </c>
-      <c r="E20" s="40">
+      <c r="E20" s="1">
         <v>7</v>
       </c>
-      <c r="F20" s="40">
-        <v>5</v>
-      </c>
-      <c r="G20" s="40">
-        <v>5</v>
-      </c>
-      <c r="H20" s="40">
-        <v>5</v>
-      </c>
-      <c r="I20" s="40">
-        <v>3</v>
-      </c>
-      <c r="J20" s="40">
+      <c r="F20" s="1">
+        <v>5</v>
+      </c>
+      <c r="G20" s="1">
+        <v>5</v>
+      </c>
+      <c r="H20" s="1">
+        <v>5</v>
+      </c>
+      <c r="I20" s="1">
+        <v>3</v>
+      </c>
+      <c r="J20" s="1">
         <v>7</v>
       </c>
-      <c r="K20" s="40">
+      <c r="K20" s="1">
         <v>6</v>
       </c>
       <c r="L20" s="35"/>
@@ -1911,36 +1899,36 @@
       <c r="N20" s="18"/>
       <c r="O20" s="7"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="34"/>
       <c r="B21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="48">
-        <v>2</v>
-      </c>
-      <c r="D21" s="48">
-        <v>2</v>
-      </c>
-      <c r="E21" s="48">
-        <v>2</v>
-      </c>
-      <c r="F21" s="48">
-        <v>1</v>
-      </c>
-      <c r="G21" s="48">
-        <v>2</v>
-      </c>
-      <c r="H21" s="48">
-        <v>1</v>
-      </c>
-      <c r="I21" s="48">
-        <v>1</v>
-      </c>
-      <c r="J21" s="48">
-        <v>1</v>
-      </c>
-      <c r="K21" s="49">
+      <c r="C21" s="41">
+        <v>2</v>
+      </c>
+      <c r="D21" s="41">
+        <v>2</v>
+      </c>
+      <c r="E21" s="41">
+        <v>2</v>
+      </c>
+      <c r="F21" s="41">
+        <v>1</v>
+      </c>
+      <c r="G21" s="41">
+        <v>2</v>
+      </c>
+      <c r="H21" s="41">
+        <v>1</v>
+      </c>
+      <c r="I21" s="41">
+        <v>1</v>
+      </c>
+      <c r="J21" s="41">
+        <v>1</v>
+      </c>
+      <c r="K21" s="42">
         <v>2</v>
       </c>
       <c r="L21" s="35">
@@ -1951,7 +1939,7 @@
       <c r="N21" s="12"/>
       <c r="O21" s="10"/>
     </row>
-    <row r="22" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="36"/>
       <c r="B22" s="3" t="s">
         <v>8</v>
@@ -1960,35 +1948,35 @@
         <f>C20-C21</f>
         <v>3</v>
       </c>
-      <c r="D22" s="50">
+      <c r="D22" s="43">
         <f t="shared" ref="D22:K22" si="5">D20-D21</f>
         <v>5</v>
       </c>
-      <c r="E22" s="50">
+      <c r="E22" s="43">
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="F22" s="50">
+      <c r="F22" s="43">
         <f t="shared" si="5"/>
         <v>4</v>
       </c>
-      <c r="G22" s="50">
+      <c r="G22" s="43">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="H22" s="50">
+      <c r="H22" s="43">
         <f t="shared" si="5"/>
         <v>4</v>
       </c>
-      <c r="I22" s="50">
+      <c r="I22" s="43">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
-      <c r="J22" s="50">
+      <c r="J22" s="43">
         <f t="shared" si="5"/>
         <v>6</v>
       </c>
-      <c r="K22" s="50">
+      <c r="K22" s="43">
         <f t="shared" si="5"/>
         <v>4</v>
       </c>
@@ -1997,38 +1985,38 @@
       <c r="N22" s="19"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="32" t="s">
         <v>12</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="40">
-        <v>5</v>
-      </c>
-      <c r="D23" s="40">
-        <v>6</v>
-      </c>
-      <c r="E23" s="40">
-        <v>6</v>
-      </c>
-      <c r="F23" s="40">
-        <v>4</v>
-      </c>
-      <c r="G23" s="40">
-        <v>4</v>
-      </c>
-      <c r="H23" s="40">
-        <v>6</v>
-      </c>
-      <c r="I23" s="40">
-        <v>4</v>
-      </c>
-      <c r="J23" s="40">
-        <v>5</v>
-      </c>
-      <c r="K23" s="40">
+      <c r="C23" s="1">
+        <v>5</v>
+      </c>
+      <c r="D23" s="1">
+        <v>6</v>
+      </c>
+      <c r="E23" s="1">
+        <v>6</v>
+      </c>
+      <c r="F23" s="1">
+        <v>4</v>
+      </c>
+      <c r="G23" s="1">
+        <v>4</v>
+      </c>
+      <c r="H23" s="1">
+        <v>6</v>
+      </c>
+      <c r="I23" s="1">
+        <v>4</v>
+      </c>
+      <c r="J23" s="1">
+        <v>5</v>
+      </c>
+      <c r="K23" s="1">
         <v>9</v>
       </c>
       <c r="L23" s="35"/>
@@ -2036,36 +2024,36 @@
       <c r="N23" s="18"/>
       <c r="O23" s="7"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="34"/>
       <c r="B24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="48">
-        <v>1</v>
-      </c>
-      <c r="D24" s="48">
-        <v>1</v>
-      </c>
-      <c r="E24" s="48">
-        <v>1</v>
-      </c>
-      <c r="F24" s="48">
-        <v>1</v>
-      </c>
-      <c r="G24" s="48">
-        <v>1</v>
-      </c>
-      <c r="H24" s="48">
-        <v>1</v>
-      </c>
-      <c r="I24" s="48">
-        <v>1</v>
-      </c>
-      <c r="J24" s="48">
-        <v>1</v>
-      </c>
-      <c r="K24" s="49">
+      <c r="C24" s="41">
+        <v>1</v>
+      </c>
+      <c r="D24" s="41">
+        <v>1</v>
+      </c>
+      <c r="E24" s="41">
+        <v>1</v>
+      </c>
+      <c r="F24" s="41">
+        <v>1</v>
+      </c>
+      <c r="G24" s="41">
+        <v>1</v>
+      </c>
+      <c r="H24" s="41">
+        <v>1</v>
+      </c>
+      <c r="I24" s="41">
+        <v>1</v>
+      </c>
+      <c r="J24" s="41">
+        <v>1</v>
+      </c>
+      <c r="K24" s="42">
         <v>1</v>
       </c>
       <c r="L24" s="35">
@@ -2076,44 +2064,44 @@
       <c r="N24" s="12"/>
       <c r="O24" s="10"/>
     </row>
-    <row r="25" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="36"/>
       <c r="B25" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="50">
+      <c r="C25" s="43">
         <f>C23-C24</f>
         <v>4</v>
       </c>
-      <c r="D25" s="50">
+      <c r="D25" s="43">
         <f t="shared" ref="D25:K25" si="6">D23-D24</f>
         <v>5</v>
       </c>
-      <c r="E25" s="50">
+      <c r="E25" s="43">
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="F25" s="50">
+      <c r="F25" s="43">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="G25" s="50">
+      <c r="G25" s="43">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="H25" s="50">
+      <c r="H25" s="43">
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="I25" s="50">
+      <c r="I25" s="43">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="J25" s="50">
+      <c r="J25" s="43">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="K25" s="50">
+      <c r="K25" s="43">
         <f t="shared" si="6"/>
         <v>8</v>
       </c>
@@ -2122,38 +2110,38 @@
       <c r="N25" s="19"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="32" t="s">
         <v>14</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="40">
-        <v>5</v>
-      </c>
-      <c r="D26" s="40">
-        <v>5</v>
-      </c>
-      <c r="E26" s="40">
-        <v>5</v>
-      </c>
-      <c r="F26" s="40">
-        <v>4</v>
-      </c>
-      <c r="G26" s="40">
-        <v>6</v>
-      </c>
-      <c r="H26" s="40">
-        <v>6</v>
-      </c>
-      <c r="I26" s="40">
-        <v>4</v>
-      </c>
-      <c r="J26" s="40">
-        <v>6</v>
-      </c>
-      <c r="K26" s="40">
+      <c r="C26" s="1">
+        <v>5</v>
+      </c>
+      <c r="D26" s="1">
+        <v>5</v>
+      </c>
+      <c r="E26" s="1">
+        <v>5</v>
+      </c>
+      <c r="F26" s="1">
+        <v>4</v>
+      </c>
+      <c r="G26" s="1">
+        <v>6</v>
+      </c>
+      <c r="H26" s="1">
+        <v>6</v>
+      </c>
+      <c r="I26" s="1">
+        <v>4</v>
+      </c>
+      <c r="J26" s="1">
+        <v>6</v>
+      </c>
+      <c r="K26" s="1">
         <v>5</v>
       </c>
       <c r="L26" s="35"/>
@@ -2161,36 +2149,36 @@
       <c r="N26" s="18"/>
       <c r="O26" s="7"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="34"/>
       <c r="B27" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="48">
-        <v>1</v>
-      </c>
-      <c r="D27" s="48">
-        <v>2</v>
-      </c>
-      <c r="E27" s="48">
-        <v>2</v>
-      </c>
-      <c r="F27" s="48">
-        <v>1</v>
-      </c>
-      <c r="G27" s="48">
-        <v>1</v>
-      </c>
-      <c r="H27" s="48">
-        <v>1</v>
-      </c>
-      <c r="I27" s="48">
-        <v>1</v>
-      </c>
-      <c r="J27" s="48">
-        <v>1</v>
-      </c>
-      <c r="K27" s="49">
+      <c r="C27" s="41">
+        <v>1</v>
+      </c>
+      <c r="D27" s="41">
+        <v>2</v>
+      </c>
+      <c r="E27" s="41">
+        <v>2</v>
+      </c>
+      <c r="F27" s="41">
+        <v>1</v>
+      </c>
+      <c r="G27" s="41">
+        <v>1</v>
+      </c>
+      <c r="H27" s="41">
+        <v>1</v>
+      </c>
+      <c r="I27" s="41">
+        <v>1</v>
+      </c>
+      <c r="J27" s="41">
+        <v>1</v>
+      </c>
+      <c r="K27" s="42">
         <v>2</v>
       </c>
       <c r="L27" s="35">
@@ -2201,12 +2189,12 @@
       <c r="N27" s="12"/>
       <c r="O27" s="10"/>
     </row>
-    <row r="28" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="36"/>
       <c r="B28" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="50">
+      <c r="C28" s="43">
         <f>C26-C27</f>
         <v>4</v>
       </c>
@@ -2218,23 +2206,23 @@
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="F28" s="50">
+      <c r="F28" s="43">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="G28" s="50">
+      <c r="G28" s="43">
         <f t="shared" si="7"/>
         <v>5</v>
       </c>
-      <c r="H28" s="50">
+      <c r="H28" s="43">
         <f t="shared" si="7"/>
         <v>5</v>
       </c>
-      <c r="I28" s="50">
+      <c r="I28" s="43">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="J28" s="50">
+      <c r="J28" s="43">
         <f t="shared" si="7"/>
         <v>5</v>
       </c>
@@ -2253,38 +2241,38 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="32" t="s">
         <v>9</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="40">
-        <v>5</v>
-      </c>
-      <c r="D29" s="40">
-        <v>5</v>
-      </c>
-      <c r="E29" s="40">
-        <v>4</v>
-      </c>
-      <c r="F29" s="40">
-        <v>4</v>
-      </c>
-      <c r="G29" s="40">
-        <v>6</v>
-      </c>
-      <c r="H29" s="40">
-        <v>4</v>
-      </c>
-      <c r="I29" s="40">
-        <v>3</v>
-      </c>
-      <c r="J29" s="40">
-        <v>4</v>
-      </c>
-      <c r="K29" s="40">
+      <c r="C29" s="1">
+        <v>5</v>
+      </c>
+      <c r="D29" s="1">
+        <v>5</v>
+      </c>
+      <c r="E29" s="1">
+        <v>4</v>
+      </c>
+      <c r="F29" s="1">
+        <v>4</v>
+      </c>
+      <c r="G29" s="1">
+        <v>6</v>
+      </c>
+      <c r="H29" s="1">
+        <v>4</v>
+      </c>
+      <c r="I29" s="1">
+        <v>3</v>
+      </c>
+      <c r="J29" s="1">
+        <v>4</v>
+      </c>
+      <c r="K29" s="1">
         <v>5</v>
       </c>
       <c r="L29" s="35"/>
@@ -2292,32 +2280,32 @@
       <c r="N29" s="18"/>
       <c r="O29" s="7"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="34"/>
       <c r="B30" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="48">
-        <v>1</v>
-      </c>
-      <c r="D30" s="48">
-        <v>1</v>
-      </c>
-      <c r="E30" s="48">
-        <v>1</v>
-      </c>
-      <c r="F30" s="48"/>
-      <c r="G30" s="48">
-        <v>1</v>
-      </c>
-      <c r="H30" s="48">
-        <v>1</v>
-      </c>
-      <c r="I30" s="48"/>
-      <c r="J30" s="48">
-        <v>1</v>
-      </c>
-      <c r="K30" s="49">
+      <c r="C30" s="41">
+        <v>1</v>
+      </c>
+      <c r="D30" s="41">
+        <v>1</v>
+      </c>
+      <c r="E30" s="41">
+        <v>1</v>
+      </c>
+      <c r="F30" s="41"/>
+      <c r="G30" s="41">
+        <v>1</v>
+      </c>
+      <c r="H30" s="41">
+        <v>1</v>
+      </c>
+      <c r="I30" s="41"/>
+      <c r="J30" s="41">
+        <v>1</v>
+      </c>
+      <c r="K30" s="42">
         <v>1</v>
       </c>
       <c r="L30" s="35">
@@ -2328,16 +2316,16 @@
       <c r="N30" s="12"/>
       <c r="O30" s="10"/>
     </row>
-    <row r="31" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="36"/>
       <c r="B31" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="50">
+      <c r="C31" s="43">
         <f>C29-C30</f>
         <v>4</v>
       </c>
-      <c r="D31" s="50">
+      <c r="D31" s="43">
         <f t="shared" ref="D31:K31" si="8">D29-D30</f>
         <v>4</v>
       </c>
@@ -2345,11 +2333,11 @@
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
-      <c r="F31" s="50">
+      <c r="F31" s="43">
         <f t="shared" si="8"/>
         <v>4</v>
       </c>
-      <c r="G31" s="50">
+      <c r="G31" s="43">
         <f t="shared" si="8"/>
         <v>5</v>
       </c>
@@ -2357,7 +2345,7 @@
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
-      <c r="I31" s="50">
+      <c r="I31" s="43">
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
@@ -2365,7 +2353,7 @@
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
-      <c r="K31" s="50">
+      <c r="K31" s="43">
         <f t="shared" si="8"/>
         <v>4</v>
       </c>
@@ -2374,38 +2362,38 @@
       <c r="N31" s="19"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="1:15" ht="15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="32" t="s">
         <v>11</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="40">
-        <v>4</v>
-      </c>
-      <c r="D32" s="40">
-        <v>6</v>
-      </c>
-      <c r="E32" s="40">
-        <v>4</v>
-      </c>
-      <c r="F32" s="40">
-        <v>4</v>
-      </c>
-      <c r="G32" s="40">
-        <v>5</v>
-      </c>
-      <c r="H32" s="40">
-        <v>4</v>
-      </c>
-      <c r="I32" s="41">
-        <v>2</v>
-      </c>
-      <c r="J32" s="40">
-        <v>4</v>
-      </c>
-      <c r="K32" s="40">
+      <c r="C32" s="1">
+        <v>4</v>
+      </c>
+      <c r="D32" s="1">
+        <v>6</v>
+      </c>
+      <c r="E32" s="1">
+        <v>4</v>
+      </c>
+      <c r="F32" s="1">
+        <v>4</v>
+      </c>
+      <c r="G32" s="1">
+        <v>5</v>
+      </c>
+      <c r="H32" s="1">
+        <v>4</v>
+      </c>
+      <c r="I32" s="52">
+        <v>2</v>
+      </c>
+      <c r="J32" s="1">
+        <v>4</v>
+      </c>
+      <c r="K32" s="1">
         <v>6</v>
       </c>
       <c r="L32" s="35"/>
@@ -2413,34 +2401,34 @@
       <c r="N32" s="18"/>
       <c r="O32" s="7"/>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="34"/>
       <c r="B33" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C33" s="48">
-        <v>1</v>
-      </c>
-      <c r="D33" s="48">
-        <v>1</v>
-      </c>
-      <c r="E33" s="48">
-        <v>1</v>
-      </c>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48">
-        <v>1</v>
-      </c>
-      <c r="H33" s="48">
-        <v>1</v>
-      </c>
-      <c r="I33" s="48">
-        <v>1</v>
-      </c>
-      <c r="J33" s="48">
-        <v>1</v>
-      </c>
-      <c r="K33" s="49">
+      <c r="C33" s="41">
+        <v>1</v>
+      </c>
+      <c r="D33" s="41">
+        <v>1</v>
+      </c>
+      <c r="E33" s="41">
+        <v>1</v>
+      </c>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41">
+        <v>1</v>
+      </c>
+      <c r="H33" s="41">
+        <v>1</v>
+      </c>
+      <c r="I33" s="41">
+        <v>1</v>
+      </c>
+      <c r="J33" s="41">
+        <v>1</v>
+      </c>
+      <c r="K33" s="42">
         <v>1</v>
       </c>
       <c r="L33" s="35">
@@ -2451,7 +2439,7 @@
       <c r="N33" s="12"/>
       <c r="O33" s="10"/>
     </row>
-    <row r="34" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="36"/>
       <c r="B34" s="3" t="s">
         <v>8</v>
@@ -2460,7 +2448,7 @@
         <f>C32-C33</f>
         <v>3</v>
       </c>
-      <c r="D34" s="50">
+      <c r="D34" s="43">
         <f t="shared" ref="D34:K34" si="9">D32-D33</f>
         <v>5</v>
       </c>
@@ -2468,11 +2456,11 @@
         <f t="shared" si="9"/>
         <v>3</v>
       </c>
-      <c r="F34" s="50">
+      <c r="F34" s="43">
         <f t="shared" si="9"/>
         <v>4</v>
       </c>
-      <c r="G34" s="50">
+      <c r="G34" s="43">
         <f t="shared" si="9"/>
         <v>4</v>
       </c>
@@ -2488,7 +2476,7 @@
         <f t="shared" si="9"/>
         <v>3</v>
       </c>
-      <c r="K34" s="50">
+      <c r="K34" s="43">
         <f t="shared" si="9"/>
         <v>5</v>
       </c>
@@ -2503,7 +2491,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C35" s="4" t="s">
         <v>19</v>
       </c>
@@ -2535,20 +2523,19 @@
         <f>SUM(M7:M34)</f>
         <v>7</v>
       </c>
-      <c r="N35" s="54">
+      <c r="N35" s="46">
         <f>SUM(N7:N34)</f>
         <v>38.85</v>
       </c>
-      <c r="O35" s="42">
+      <c r="O35" s="40">
         <f>SUM(O7:O34)</f>
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D36" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E36" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>